<commit_message>
upload the new annotations files
</commit_message>
<xml_diff>
--- a/annotation/a604.xlsx
+++ b/annotation/a604.xlsx
@@ -10,6 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Mots" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Horizontales" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Verticales" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DeletedCells" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -415,7 +416,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L59"/>
+  <dimension ref="A1:O60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -451,30 +452,45 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>parent_id</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>part_id</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>part_index</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>num_sora</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>sora_name_ar</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>aya_no</t>
+        </is>
+      </c>
+      <c r="M1" t="inlineStr">
+        <is>
           <t>kalima_text</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>num_sora</t>
-        </is>
-      </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>sora_name_ar</t>
-        </is>
-      </c>
-      <c r="J1" t="inlineStr">
-        <is>
-          <t>aya_no</t>
-        </is>
-      </c>
-      <c r="K1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>kalima_text_emlaey</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>line</t>
         </is>
@@ -499,29 +515,38 @@
       <c r="F2" t="n">
         <v>1</v>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr"/>
+      <c r="I2" t="inlineStr"/>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>112.0</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>الإخلَاص</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
         <is>
           <t>قُلۡ</t>
         </is>
       </c>
-      <c r="H2" t="n">
-        <v>112</v>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>الإخلَاص</t>
-        </is>
-      </c>
-      <c r="J2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>قل</t>
         </is>
       </c>
-      <c r="L2" t="n">
-        <v>0</v>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -543,29 +568,38 @@
       <c r="F3" t="n">
         <v>2</v>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr"/>
+      <c r="I3" t="inlineStr"/>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>112.0</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>الإخلَاص</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
         <is>
           <t>هُوَ</t>
         </is>
       </c>
-      <c r="H3" t="n">
-        <v>112</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>الإخلَاص</t>
-        </is>
-      </c>
-      <c r="J3" t="n">
-        <v>1</v>
-      </c>
-      <c r="K3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>هو</t>
         </is>
       </c>
-      <c r="L3" t="n">
-        <v>0</v>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -587,29 +621,38 @@
       <c r="F4" t="n">
         <v>3</v>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr"/>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>112.0</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>الإخلَاص</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
         <is>
           <t>ٱللَّهُ</t>
         </is>
       </c>
-      <c r="H4" t="n">
-        <v>112</v>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>الإخلَاص</t>
-        </is>
-      </c>
-      <c r="J4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>الله</t>
         </is>
       </c>
-      <c r="L4" t="n">
-        <v>0</v>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -629,32 +672,17 @@
         <v>0</v>
       </c>
       <c r="F5" t="n">
-        <v>4</v>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>أَحَدٌ</t>
-        </is>
-      </c>
-      <c r="H5" t="n">
-        <v>112</v>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>الإخلَاص</t>
-        </is>
-      </c>
-      <c r="J5" t="n">
-        <v>1</v>
-      </c>
-      <c r="K5" t="inlineStr">
-        <is>
-          <t>أحد</t>
-        </is>
-      </c>
-      <c r="L5" t="n">
-        <v>0</v>
-      </c>
+        <v>63</v>
+      </c>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr"/>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr"/>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -673,36 +701,45 @@
         <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>6</v>
-      </c>
-      <c r="G6" t="inlineStr">
+        <v>5</v>
+      </c>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr"/>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>112.0</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>الإخلَاص</t>
+        </is>
+      </c>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr">
         <is>
           <t>ٱللَّهُ</t>
         </is>
       </c>
-      <c r="H6" t="n">
-        <v>112</v>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>الإخلَاص</t>
-        </is>
-      </c>
-      <c r="J6" t="n">
-        <v>2</v>
-      </c>
-      <c r="K6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>الله</t>
         </is>
       </c>
-      <c r="L6" t="n">
-        <v>0</v>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="n">
-        <v>146.1900826446281</v>
+        <v>169.1922246220302</v>
       </c>
       <c r="B7" t="n">
         <v>113.2148760330578</v>
@@ -717,42 +754,57 @@
         <v>0</v>
       </c>
       <c r="F7" t="n">
-        <v>7</v>
-      </c>
-      <c r="G7" t="inlineStr">
+        <v>62</v>
+      </c>
+      <c r="G7" t="n">
+        <v>6</v>
+      </c>
+      <c r="H7" t="n">
+        <v>2</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2</v>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>112.0</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>الإخلَاص</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
         <is>
           <t>ٱلصَّمَدُ</t>
         </is>
       </c>
-      <c r="H7" t="n">
-        <v>112</v>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>الإخلَاص</t>
-        </is>
-      </c>
-      <c r="J7" t="n">
-        <v>2</v>
-      </c>
-      <c r="K7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>الصمد</t>
         </is>
       </c>
-      <c r="L7" t="n">
-        <v>0</v>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="n">
-        <v>80.23966942148759</v>
+        <v>146.1900826446281</v>
       </c>
       <c r="B8" t="n">
         <v>113.2148760330578</v>
       </c>
       <c r="C8" t="n">
-        <v>107.7190082644628</v>
+        <v>169.1922246220302</v>
       </c>
       <c r="D8" t="n">
         <v>161.5785123966942</v>
@@ -761,42 +813,57 @@
         <v>0</v>
       </c>
       <c r="F8" t="n">
-        <v>9</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>لَمۡ</t>
-        </is>
+        <v>61</v>
+      </c>
+      <c r="G8" t="n">
+        <v>6</v>
       </c>
       <c r="H8" t="n">
-        <v>112</v>
-      </c>
-      <c r="I8" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="I8" t="n">
+        <v>1</v>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>112.0</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
         <is>
           <t>الإخلَاص</t>
         </is>
       </c>
-      <c r="J8" t="n">
-        <v>3</v>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>لم</t>
-        </is>
-      </c>
-      <c r="L8" t="n">
-        <v>0</v>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>ٱلصَّمَدُ</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>الصمد</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="n">
-        <v>9.892561983471074</v>
+        <v>80.23966942148759</v>
       </c>
       <c r="B9" t="n">
         <v>113.2148760330578</v>
       </c>
       <c r="C9" t="n">
-        <v>80.23966942148759</v>
+        <v>107.7190082644628</v>
       </c>
       <c r="D9" t="n">
         <v>161.5785123966942</v>
@@ -805,86 +872,104 @@
         <v>0</v>
       </c>
       <c r="F9" t="n">
-        <v>10</v>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>يَلِدۡ</t>
-        </is>
-      </c>
-      <c r="H9" t="n">
-        <v>112</v>
-      </c>
-      <c r="I9" t="inlineStr">
+        <v>7</v>
+      </c>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr"/>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>112.0</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
         <is>
           <t>الإخلَاص</t>
         </is>
       </c>
-      <c r="J9" t="n">
-        <v>3</v>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>يلد</t>
-        </is>
-      </c>
-      <c r="L9" t="n">
-        <v>0</v>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>لَمۡ</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>لم</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="n">
-        <v>458.3553719008264</v>
+        <v>9.892561983471074</v>
       </c>
       <c r="B10" t="n">
+        <v>113.2148760330578</v>
+      </c>
+      <c r="C10" t="n">
+        <v>80.23966942148759</v>
+      </c>
+      <c r="D10" t="n">
         <v>161.5785123966942</v>
       </c>
-      <c r="C10" t="n">
-        <v>503.4214876033058</v>
-      </c>
-      <c r="D10" t="n">
-        <v>217.6363636363636</v>
-      </c>
       <c r="E10" t="b">
         <v>0</v>
       </c>
       <c r="F10" t="n">
-        <v>11</v>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>وَلَمۡ</t>
-        </is>
-      </c>
-      <c r="H10" t="n">
-        <v>112</v>
-      </c>
-      <c r="I10" t="inlineStr">
+        <v>8</v>
+      </c>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr"/>
+      <c r="I10" t="inlineStr"/>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>112.0</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
         <is>
           <t>الإخلَاص</t>
         </is>
       </c>
-      <c r="J10" t="n">
-        <v>3</v>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>ولم</t>
-        </is>
-      </c>
-      <c r="L10" t="n">
-        <v>0</v>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>يَلِدۡ</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>يلد</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="n">
-        <v>402.297520661157</v>
+        <v>458.3553719008264</v>
       </c>
       <c r="B11" t="n">
         <v>161.5785123966942</v>
       </c>
       <c r="C11" t="n">
-        <v>458.3553719008264</v>
+        <v>503.4214876033058</v>
       </c>
       <c r="D11" t="n">
         <v>217.6363636363636</v>
@@ -893,42 +978,51 @@
         <v>0</v>
       </c>
       <c r="F11" t="n">
-        <v>12</v>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>يُولَدۡ</t>
-        </is>
-      </c>
-      <c r="H11" t="n">
-        <v>112</v>
-      </c>
-      <c r="I11" t="inlineStr">
+        <v>9</v>
+      </c>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr"/>
+      <c r="I11" t="inlineStr"/>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>112.0</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
         <is>
           <t>الإخلَاص</t>
         </is>
       </c>
-      <c r="J11" t="n">
-        <v>3</v>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>يولد</t>
-        </is>
-      </c>
-      <c r="L11" t="n">
-        <v>0</v>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>وَلَمۡ</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>ولم</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="n">
-        <v>326.4545454545454</v>
+        <v>402.297520661157</v>
       </c>
       <c r="B12" t="n">
         <v>161.5785123966942</v>
       </c>
       <c r="C12" t="n">
-        <v>367.1239669421487</v>
+        <v>458.3553719008264</v>
       </c>
       <c r="D12" t="n">
         <v>217.6363636363636</v>
@@ -937,42 +1031,51 @@
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>15</v>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>وَلَمۡ</t>
-        </is>
-      </c>
-      <c r="H12" t="n">
-        <v>112</v>
-      </c>
-      <c r="I12" t="inlineStr">
+        <v>10</v>
+      </c>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr"/>
+      <c r="I12" t="inlineStr"/>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>112.0</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
         <is>
           <t>الإخلَاص</t>
         </is>
       </c>
-      <c r="J12" t="n">
-        <v>4</v>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>ولم</t>
-        </is>
-      </c>
-      <c r="L12" t="n">
-        <v>0</v>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>يُولَدۡ</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>يولد</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="n">
-        <v>238.5206611570248</v>
+        <v>326.4545454545454</v>
       </c>
       <c r="B13" t="n">
         <v>161.5785123966942</v>
       </c>
       <c r="C13" t="n">
-        <v>326.4545454545454</v>
+        <v>367.1239669421487</v>
       </c>
       <c r="D13" t="n">
         <v>217.6363636363636</v>
@@ -981,42 +1084,51 @@
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>16</v>
-      </c>
-      <c r="G13" t="inlineStr">
-        <is>
-          <t>يَكُن</t>
-        </is>
-      </c>
-      <c r="H13" t="n">
-        <v>112</v>
-      </c>
-      <c r="I13" t="inlineStr">
+        <v>11</v>
+      </c>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr"/>
+      <c r="I13" t="inlineStr"/>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>112.0</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
         <is>
           <t>الإخلَاص</t>
         </is>
       </c>
-      <c r="J13" t="n">
-        <v>4</v>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>يكن</t>
-        </is>
-      </c>
-      <c r="L13" t="n">
-        <v>0</v>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>وَلَمۡ</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>ولم</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="n">
-        <v>212.1404958677686</v>
+        <v>238.5206611570248</v>
       </c>
       <c r="B14" t="n">
         <v>161.5785123966942</v>
       </c>
       <c r="C14" t="n">
-        <v>238.5206611570248</v>
+        <v>326.4545454545454</v>
       </c>
       <c r="D14" t="n">
         <v>217.6363636363636</v>
@@ -1025,42 +1137,51 @@
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>17</v>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>لَّهُۥ</t>
-        </is>
-      </c>
-      <c r="H14" t="n">
-        <v>112</v>
-      </c>
-      <c r="I14" t="inlineStr">
+        <v>12</v>
+      </c>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr"/>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>112.0</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
         <is>
           <t>الإخلَاص</t>
         </is>
       </c>
-      <c r="J14" t="n">
-        <v>4</v>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>له</t>
-        </is>
-      </c>
-      <c r="L14" t="n">
-        <v>0</v>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>يَكُن</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>يكن</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="n">
-        <v>123.1074380165289</v>
+        <v>212.1404958677686</v>
       </c>
       <c r="B15" t="n">
         <v>161.5785123966942</v>
       </c>
       <c r="C15" t="n">
-        <v>212.1404958677686</v>
+        <v>238.5206611570248</v>
       </c>
       <c r="D15" t="n">
         <v>217.6363636363636</v>
@@ -1069,42 +1190,51 @@
         <v>0</v>
       </c>
       <c r="F15" t="n">
-        <v>18</v>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>كُفُوًا</t>
-        </is>
-      </c>
-      <c r="H15" t="n">
-        <v>112</v>
-      </c>
-      <c r="I15" t="inlineStr">
+        <v>13</v>
+      </c>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr"/>
+      <c r="I15" t="inlineStr"/>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>112.0</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
         <is>
           <t>الإخلَاص</t>
         </is>
       </c>
-      <c r="J15" t="n">
-        <v>4</v>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>كفوا</t>
-        </is>
-      </c>
-      <c r="L15" t="n">
-        <v>0</v>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>لَّهُۥ</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>له</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="n">
-        <v>53.8595041322314</v>
+        <v>123.1074380165289</v>
       </c>
       <c r="B16" t="n">
         <v>161.5785123966942</v>
       </c>
       <c r="C16" t="n">
-        <v>123.1074380165289</v>
+        <v>212.1404958677686</v>
       </c>
       <c r="D16" t="n">
         <v>217.6363636363636</v>
@@ -1113,86 +1243,104 @@
         <v>0</v>
       </c>
       <c r="F16" t="n">
-        <v>19</v>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>أَحَدُۢ</t>
-        </is>
-      </c>
-      <c r="H16" t="n">
-        <v>112</v>
-      </c>
-      <c r="I16" t="inlineStr">
+        <v>14</v>
+      </c>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr"/>
+      <c r="I16" t="inlineStr"/>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>112.0</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
         <is>
           <t>الإخلَاص</t>
         </is>
       </c>
-      <c r="J16" t="n">
-        <v>4</v>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>أحد</t>
-        </is>
-      </c>
-      <c r="L16" t="n">
-        <v>0</v>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>كُفُوًا</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>كفوا</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="n">
-        <v>470.4462809917355</v>
+        <v>53.8595041322314</v>
       </c>
       <c r="B17" t="n">
-        <v>324.2561983471074</v>
+        <v>161.5785123966942</v>
       </c>
       <c r="C17" t="n">
-        <v>500.1239669421487</v>
+        <v>123.1074380165289</v>
       </c>
       <c r="D17" t="n">
-        <v>375.9173553719008</v>
+        <v>217.6363636363636</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
       </c>
       <c r="F17" t="n">
-        <v>20</v>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>قُلۡ</t>
-        </is>
-      </c>
-      <c r="H17" t="n">
-        <v>113</v>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>الفَلَق</t>
-        </is>
-      </c>
-      <c r="J17" t="n">
-        <v>1</v>
+        <v>15</v>
+      </c>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr"/>
+      <c r="I17" t="inlineStr"/>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>112.0</t>
+        </is>
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>قل</t>
-        </is>
-      </c>
-      <c r="L17" t="n">
-        <v>0</v>
+          <t>الإخلَاص</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>أَحَدُۢ</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>أحد</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="n">
-        <v>422.0826446280992</v>
+        <v>470.4462809917355</v>
       </c>
       <c r="B18" t="n">
         <v>324.2561983471074</v>
       </c>
       <c r="C18" t="n">
-        <v>470.4462809917355</v>
+        <v>500.1239669421487</v>
       </c>
       <c r="D18" t="n">
         <v>375.9173553719008</v>
@@ -1201,42 +1349,51 @@
         <v>0</v>
       </c>
       <c r="F18" t="n">
-        <v>21</v>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>أَعُوذُ</t>
-        </is>
-      </c>
-      <c r="H18" t="n">
-        <v>113</v>
-      </c>
-      <c r="I18" t="inlineStr">
+        <v>16</v>
+      </c>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr"/>
+      <c r="I18" t="inlineStr"/>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>113.0</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
         <is>
           <t>الفَلَق</t>
         </is>
       </c>
-      <c r="J18" t="n">
-        <v>1</v>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>أعوذ</t>
-        </is>
-      </c>
-      <c r="L18" t="n">
-        <v>0</v>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>قُلۡ</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>قل</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="n">
-        <v>366.0247933884297</v>
+        <v>422.0826446280992</v>
       </c>
       <c r="B19" t="n">
         <v>324.2561983471074</v>
       </c>
       <c r="C19" t="n">
-        <v>422.0826446280992</v>
+        <v>470.4462809917355</v>
       </c>
       <c r="D19" t="n">
         <v>375.9173553719008</v>
@@ -1245,42 +1402,51 @@
         <v>0</v>
       </c>
       <c r="F19" t="n">
-        <v>22</v>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>بِرَبِّ</t>
-        </is>
-      </c>
-      <c r="H19" t="n">
-        <v>113</v>
-      </c>
-      <c r="I19" t="inlineStr">
+        <v>17</v>
+      </c>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr"/>
+      <c r="I19" t="inlineStr"/>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>113.0</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
         <is>
           <t>الفَلَق</t>
         </is>
       </c>
-      <c r="J19" t="n">
-        <v>1</v>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>برب</t>
-        </is>
-      </c>
-      <c r="L19" t="n">
-        <v>0</v>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>أَعُوذُ</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>أعوذ</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="n">
-        <v>300.0743801652892</v>
+        <v>366.0247933884297</v>
       </c>
       <c r="B20" t="n">
         <v>324.2561983471074</v>
       </c>
       <c r="C20" t="n">
-        <v>366.0247933884297</v>
+        <v>422.0826446280992</v>
       </c>
       <c r="D20" t="n">
         <v>375.9173553719008</v>
@@ -1289,42 +1455,51 @@
         <v>0</v>
       </c>
       <c r="F20" t="n">
-        <v>23</v>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>ٱلۡفَلَقِ</t>
-        </is>
-      </c>
-      <c r="H20" t="n">
-        <v>113</v>
-      </c>
-      <c r="I20" t="inlineStr">
+        <v>18</v>
+      </c>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr"/>
+      <c r="I20" t="inlineStr"/>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>113.0</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
         <is>
           <t>الفَلَق</t>
         </is>
       </c>
-      <c r="J20" t="n">
-        <v>1</v>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>الفلق</t>
-        </is>
-      </c>
-      <c r="L20" t="n">
-        <v>0</v>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>بِرَبِّ</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>برب</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="n">
-        <v>233.0247933884297</v>
+        <v>300.0743801652892</v>
       </c>
       <c r="B21" t="n">
         <v>324.2561983471074</v>
       </c>
       <c r="C21" t="n">
-        <v>266</v>
+        <v>366.0247933884297</v>
       </c>
       <c r="D21" t="n">
         <v>375.9173553719008</v>
@@ -1333,42 +1508,51 @@
         <v>0</v>
       </c>
       <c r="F21" t="n">
-        <v>25</v>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>مِن</t>
-        </is>
-      </c>
-      <c r="H21" t="n">
-        <v>113</v>
-      </c>
-      <c r="I21" t="inlineStr">
+        <v>19</v>
+      </c>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr"/>
+      <c r="I21" t="inlineStr"/>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>113.0</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
         <is>
           <t>الفَلَق</t>
         </is>
       </c>
-      <c r="J21" t="n">
-        <v>2</v>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>من</t>
-        </is>
-      </c>
-      <c r="L21" t="n">
-        <v>0</v>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>ٱلۡفَلَقِ</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>الفلق</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="n">
-        <v>203.3471074380165</v>
+        <v>233.0247933884297</v>
       </c>
       <c r="B22" t="n">
         <v>324.2561983471074</v>
       </c>
       <c r="C22" t="n">
-        <v>233.0247933884297</v>
+        <v>266</v>
       </c>
       <c r="D22" t="n">
         <v>375.9173553719008</v>
@@ -1377,42 +1561,51 @@
         <v>0</v>
       </c>
       <c r="F22" t="n">
-        <v>26</v>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>شَرِّ</t>
-        </is>
-      </c>
-      <c r="H22" t="n">
-        <v>113</v>
-      </c>
-      <c r="I22" t="inlineStr">
+        <v>20</v>
+      </c>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr"/>
+      <c r="I22" t="inlineStr"/>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>113.0</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
         <is>
           <t>الفَلَق</t>
         </is>
       </c>
-      <c r="J22" t="n">
-        <v>2</v>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>شر</t>
-        </is>
-      </c>
-      <c r="L22" t="n">
-        <v>0</v>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>مِن</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>من</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
-        <v>184.6611570247934</v>
+        <v>203.3471074380165</v>
       </c>
       <c r="B23" t="n">
         <v>324.2561983471074</v>
       </c>
       <c r="C23" t="n">
-        <v>203.3471074380165</v>
+        <v>233.0247933884297</v>
       </c>
       <c r="D23" t="n">
         <v>375.9173553719008</v>
@@ -1421,42 +1614,51 @@
         <v>0</v>
       </c>
       <c r="F23" t="n">
-        <v>27</v>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>مَا</t>
-        </is>
-      </c>
-      <c r="H23" t="n">
-        <v>113</v>
-      </c>
-      <c r="I23" t="inlineStr">
+        <v>21</v>
+      </c>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr"/>
+      <c r="I23" t="inlineStr"/>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>113.0</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
         <is>
           <t>الفَلَق</t>
         </is>
       </c>
-      <c r="J23" t="n">
-        <v>2</v>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>ما</t>
-        </is>
-      </c>
-      <c r="L23" t="n">
-        <v>0</v>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>شَرِّ</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>شر</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
-        <v>134.099173553719</v>
+        <v>184.6611570247934</v>
       </c>
       <c r="B24" t="n">
         <v>324.2561983471074</v>
       </c>
       <c r="C24" t="n">
-        <v>184.6611570247934</v>
+        <v>203.3471074380165</v>
       </c>
       <c r="D24" t="n">
         <v>375.9173553719008</v>
@@ -1465,42 +1667,51 @@
         <v>0</v>
       </c>
       <c r="F24" t="n">
-        <v>28</v>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>خَلَقَ</t>
-        </is>
-      </c>
-      <c r="H24" t="n">
-        <v>113</v>
-      </c>
-      <c r="I24" t="inlineStr">
+        <v>22</v>
+      </c>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr"/>
+      <c r="I24" t="inlineStr"/>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>113.0</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
         <is>
           <t>الفَلَق</t>
         </is>
       </c>
-      <c r="J24" t="n">
-        <v>2</v>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>خلق</t>
-        </is>
-      </c>
-      <c r="L24" t="n">
-        <v>0</v>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>مَا</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>ما</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
-        <v>51.66115702479338</v>
+        <v>134.099173553719</v>
       </c>
       <c r="B25" t="n">
         <v>324.2561983471074</v>
       </c>
       <c r="C25" t="n">
-        <v>96.72727272727272</v>
+        <v>184.6611570247934</v>
       </c>
       <c r="D25" t="n">
         <v>375.9173553719008</v>
@@ -1509,42 +1720,51 @@
         <v>0</v>
       </c>
       <c r="F25" t="n">
-        <v>30</v>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>وَمِن</t>
-        </is>
-      </c>
-      <c r="H25" t="n">
-        <v>113</v>
-      </c>
-      <c r="I25" t="inlineStr">
+        <v>23</v>
+      </c>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr"/>
+      <c r="I25" t="inlineStr"/>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>113.0</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
         <is>
           <t>الفَلَق</t>
         </is>
       </c>
-      <c r="J25" t="n">
-        <v>3</v>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>ومن</t>
-        </is>
-      </c>
-      <c r="L25" t="n">
-        <v>0</v>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>خَلَقَ</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>خلق</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
-        <v>9.892561983471074</v>
+        <v>51.66115702479338</v>
       </c>
       <c r="B26" t="n">
         <v>324.2561983471074</v>
       </c>
       <c r="C26" t="n">
-        <v>51.66115702479338</v>
+        <v>96.72727272727272</v>
       </c>
       <c r="D26" t="n">
         <v>375.9173553719008</v>
@@ -1553,86 +1773,104 @@
         <v>0</v>
       </c>
       <c r="F26" t="n">
-        <v>31</v>
-      </c>
-      <c r="G26" t="inlineStr">
-        <is>
-          <t>شَرِّ</t>
-        </is>
-      </c>
-      <c r="H26" t="n">
-        <v>113</v>
-      </c>
-      <c r="I26" t="inlineStr">
+        <v>24</v>
+      </c>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr"/>
+      <c r="I26" t="inlineStr"/>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>113.0</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
         <is>
           <t>الفَلَق</t>
         </is>
       </c>
-      <c r="J26" t="n">
-        <v>3</v>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>شر</t>
-        </is>
-      </c>
-      <c r="L26" t="n">
-        <v>0</v>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>وَمِن</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>ومن</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
-        <v>437.4710743801652</v>
+        <v>9.892561983471074</v>
       </c>
       <c r="B27" t="n">
+        <v>324.2561983471074</v>
+      </c>
+      <c r="C27" t="n">
+        <v>51.66115702479338</v>
+      </c>
+      <c r="D27" t="n">
         <v>375.9173553719008</v>
       </c>
-      <c r="C27" t="n">
-        <v>501.2231404958677</v>
-      </c>
-      <c r="D27" t="n">
-        <v>428.6776859504132</v>
-      </c>
       <c r="E27" t="b">
         <v>0</v>
       </c>
       <c r="F27" t="n">
-        <v>32</v>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>غَاسِقٍ</t>
-        </is>
-      </c>
-      <c r="H27" t="n">
-        <v>113</v>
-      </c>
-      <c r="I27" t="inlineStr">
+        <v>25</v>
+      </c>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr"/>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>113.0</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
         <is>
           <t>الفَلَق</t>
         </is>
       </c>
-      <c r="J27" t="n">
-        <v>3</v>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>غاسق</t>
-        </is>
-      </c>
-      <c r="L27" t="n">
-        <v>0</v>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>شَرِّ</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>شر</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
-        <v>408.892561983471</v>
+        <v>437.4710743801652</v>
       </c>
       <c r="B28" t="n">
         <v>375.9173553719008</v>
       </c>
       <c r="C28" t="n">
-        <v>437.4710743801652</v>
+        <v>501.2231404958677</v>
       </c>
       <c r="D28" t="n">
         <v>428.6776859504132</v>
@@ -1641,42 +1879,51 @@
         <v>0</v>
       </c>
       <c r="F28" t="n">
-        <v>33</v>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>إِذَا</t>
-        </is>
-      </c>
-      <c r="H28" t="n">
-        <v>113</v>
-      </c>
-      <c r="I28" t="inlineStr">
+        <v>26</v>
+      </c>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr"/>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>113.0</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
         <is>
           <t>الفَلَق</t>
         </is>
       </c>
-      <c r="J28" t="n">
-        <v>3</v>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>إذا</t>
-        </is>
-      </c>
-      <c r="L28" t="n">
-        <v>0</v>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>غَاسِقٍ</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>غاسق</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
-        <v>355.0330578512396</v>
+        <v>408.892561983471</v>
       </c>
       <c r="B29" t="n">
         <v>375.9173553719008</v>
       </c>
       <c r="C29" t="n">
-        <v>408.892561983471</v>
+        <v>437.4710743801652</v>
       </c>
       <c r="D29" t="n">
         <v>428.6776859504132</v>
@@ -1685,42 +1932,51 @@
         <v>0</v>
       </c>
       <c r="F29" t="n">
-        <v>34</v>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>وَقَبَ</t>
-        </is>
-      </c>
-      <c r="H29" t="n">
-        <v>113</v>
-      </c>
-      <c r="I29" t="inlineStr">
+        <v>27</v>
+      </c>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>113.0</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
         <is>
           <t>الفَلَق</t>
         </is>
       </c>
-      <c r="J29" t="n">
-        <v>3</v>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>وقب</t>
-        </is>
-      </c>
-      <c r="L29" t="n">
-        <v>0</v>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>إِذَا</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>إذا</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
-        <v>278.0909090909091</v>
+        <v>355.0330578512396</v>
       </c>
       <c r="B30" t="n">
         <v>375.9173553719008</v>
       </c>
       <c r="C30" t="n">
-        <v>320.9586776859504</v>
+        <v>408.892561983471</v>
       </c>
       <c r="D30" t="n">
         <v>428.6776859504132</v>
@@ -1729,42 +1985,51 @@
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>36</v>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>وَمِن</t>
-        </is>
-      </c>
-      <c r="H30" t="n">
-        <v>113</v>
-      </c>
-      <c r="I30" t="inlineStr">
+        <v>28</v>
+      </c>
+      <c r="G30" t="inlineStr"/>
+      <c r="H30" t="inlineStr"/>
+      <c r="I30" t="inlineStr"/>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>113.0</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
         <is>
           <t>الفَلَق</t>
         </is>
       </c>
-      <c r="J30" t="n">
-        <v>4</v>
-      </c>
-      <c r="K30" t="inlineStr">
-        <is>
-          <t>ومن</t>
-        </is>
-      </c>
-      <c r="L30" t="n">
-        <v>0</v>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>وَقَبَ</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>وقب</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
-        <v>241.8181818181818</v>
+        <v>278.0909090909091</v>
       </c>
       <c r="B31" t="n">
         <v>375.9173553719008</v>
       </c>
       <c r="C31" t="n">
-        <v>278.0909090909091</v>
+        <v>320.9586776859504</v>
       </c>
       <c r="D31" t="n">
         <v>428.6776859504132</v>
@@ -1773,42 +2038,51 @@
         <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>37</v>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>شَرِّ</t>
-        </is>
-      </c>
-      <c r="H31" t="n">
-        <v>113</v>
-      </c>
-      <c r="I31" t="inlineStr">
+        <v>29</v>
+      </c>
+      <c r="G31" t="inlineStr"/>
+      <c r="H31" t="inlineStr"/>
+      <c r="I31" t="inlineStr"/>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>113.0</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
         <is>
           <t>الفَلَق</t>
         </is>
       </c>
-      <c r="J31" t="n">
-        <v>4</v>
-      </c>
-      <c r="K31" t="inlineStr">
-        <is>
-          <t>شر</t>
-        </is>
-      </c>
-      <c r="L31" t="n">
-        <v>0</v>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>وَمِن</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>ومن</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
-        <v>143.9917355371901</v>
+        <v>241.8181818181818</v>
       </c>
       <c r="B32" t="n">
         <v>375.9173553719008</v>
       </c>
       <c r="C32" t="n">
-        <v>241.8181818181818</v>
+        <v>278.0909090909091</v>
       </c>
       <c r="D32" t="n">
         <v>428.6776859504132</v>
@@ -1817,42 +2091,51 @@
         <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>38</v>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>ٱلنَّفَّٰثَٰتِ</t>
-        </is>
-      </c>
-      <c r="H32" t="n">
-        <v>113</v>
-      </c>
-      <c r="I32" t="inlineStr">
+        <v>30</v>
+      </c>
+      <c r="G32" t="inlineStr"/>
+      <c r="H32" t="inlineStr"/>
+      <c r="I32" t="inlineStr"/>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>113.0</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
         <is>
           <t>الفَلَق</t>
         </is>
       </c>
-      <c r="J32" t="n">
-        <v>4</v>
-      </c>
-      <c r="K32" t="inlineStr">
-        <is>
-          <t>النفاثات</t>
-        </is>
-      </c>
-      <c r="L32" t="n">
-        <v>0</v>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>شَرِّ</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>شر</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
-        <v>117.6115702479339</v>
+        <v>143.9917355371901</v>
       </c>
       <c r="B33" t="n">
         <v>375.9173553719008</v>
       </c>
       <c r="C33" t="n">
-        <v>143.9917355371901</v>
+        <v>241.8181818181818</v>
       </c>
       <c r="D33" t="n">
         <v>428.6776859504132</v>
@@ -1861,42 +2144,51 @@
         <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>39</v>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>فِي</t>
-        </is>
-      </c>
-      <c r="H33" t="n">
-        <v>113</v>
-      </c>
-      <c r="I33" t="inlineStr">
+        <v>31</v>
+      </c>
+      <c r="G33" t="inlineStr"/>
+      <c r="H33" t="inlineStr"/>
+      <c r="I33" t="inlineStr"/>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>113.0</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
         <is>
           <t>الفَلَق</t>
         </is>
       </c>
-      <c r="J33" t="n">
-        <v>4</v>
-      </c>
-      <c r="K33" t="inlineStr">
-        <is>
-          <t>في</t>
-        </is>
-      </c>
-      <c r="L33" t="n">
-        <v>0</v>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>ٱلنَّفَّٰثَٰتِ</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>النفاثات</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
-        <v>47.26446280991735</v>
+        <v>117.6115702479339</v>
       </c>
       <c r="B34" t="n">
         <v>375.9173553719008</v>
       </c>
       <c r="C34" t="n">
-        <v>117.6115702479339</v>
+        <v>143.9917355371901</v>
       </c>
       <c r="D34" t="n">
         <v>428.6776859504132</v>
@@ -1905,86 +2197,104 @@
         <v>0</v>
       </c>
       <c r="F34" t="n">
-        <v>40</v>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>ٱلۡعُقَدِ</t>
-        </is>
-      </c>
-      <c r="H34" t="n">
-        <v>113</v>
-      </c>
-      <c r="I34" t="inlineStr">
+        <v>32</v>
+      </c>
+      <c r="G34" t="inlineStr"/>
+      <c r="H34" t="inlineStr"/>
+      <c r="I34" t="inlineStr"/>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>113.0</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
         <is>
           <t>الفَلَق</t>
         </is>
       </c>
-      <c r="J34" t="n">
-        <v>4</v>
-      </c>
-      <c r="K34" t="inlineStr">
-        <is>
-          <t>العقد</t>
-        </is>
-      </c>
-      <c r="L34" t="n">
-        <v>0</v>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>فِي</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>في</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
-        <v>352.8347107438016</v>
+        <v>47.26446280991735</v>
       </c>
       <c r="B35" t="n">
+        <v>375.9173553719008</v>
+      </c>
+      <c r="C35" t="n">
+        <v>117.6115702479339</v>
+      </c>
+      <c r="D35" t="n">
         <v>428.6776859504132</v>
       </c>
-      <c r="C35" t="n">
-        <v>402.297520661157</v>
-      </c>
-      <c r="D35" t="n">
-        <v>478.1404958677685</v>
-      </c>
       <c r="E35" t="b">
         <v>0</v>
       </c>
       <c r="F35" t="n">
-        <v>41</v>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>وَمِن</t>
-        </is>
-      </c>
-      <c r="H35" t="n">
-        <v>113</v>
-      </c>
-      <c r="I35" t="inlineStr">
+        <v>33</v>
+      </c>
+      <c r="G35" t="inlineStr"/>
+      <c r="H35" t="inlineStr"/>
+      <c r="I35" t="inlineStr"/>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>113.0</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
         <is>
           <t>الفَلَق</t>
         </is>
       </c>
-      <c r="J35" t="n">
-        <v>5</v>
-      </c>
-      <c r="K35" t="inlineStr">
-        <is>
-          <t>ومن</t>
-        </is>
-      </c>
-      <c r="L35" t="n">
-        <v>0</v>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>ٱلۡعُقَدِ</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>العقد</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
-        <v>308.8677685950413</v>
+        <v>352.8347107438016</v>
       </c>
       <c r="B36" t="n">
         <v>428.6776859504132</v>
       </c>
       <c r="C36" t="n">
-        <v>352.8347107438016</v>
+        <v>402.297520661157</v>
       </c>
       <c r="D36" t="n">
         <v>478.1404958677685</v>
@@ -1993,42 +2303,51 @@
         <v>0</v>
       </c>
       <c r="F36" t="n">
-        <v>42</v>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>شَرِّ</t>
-        </is>
-      </c>
-      <c r="H36" t="n">
-        <v>113</v>
-      </c>
-      <c r="I36" t="inlineStr">
+        <v>34</v>
+      </c>
+      <c r="G36" t="inlineStr"/>
+      <c r="H36" t="inlineStr"/>
+      <c r="I36" t="inlineStr"/>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>113.0</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
         <is>
           <t>الفَلَق</t>
         </is>
       </c>
-      <c r="J36" t="n">
-        <v>5</v>
-      </c>
-      <c r="K36" t="inlineStr">
-        <is>
-          <t>شر</t>
-        </is>
-      </c>
-      <c r="L36" t="n">
-        <v>0</v>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>وَمِن</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>ومن</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
-        <v>245.1157024793388</v>
+        <v>308.8677685950413</v>
       </c>
       <c r="B37" t="n">
         <v>428.6776859504132</v>
       </c>
       <c r="C37" t="n">
-        <v>308.8677685950413</v>
+        <v>352.8347107438016</v>
       </c>
       <c r="D37" t="n">
         <v>478.1404958677685</v>
@@ -2037,42 +2356,51 @@
         <v>0</v>
       </c>
       <c r="F37" t="n">
-        <v>43</v>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>حَاسِدٍ</t>
-        </is>
-      </c>
-      <c r="H37" t="n">
-        <v>113</v>
-      </c>
-      <c r="I37" t="inlineStr">
+        <v>35</v>
+      </c>
+      <c r="G37" t="inlineStr"/>
+      <c r="H37" t="inlineStr"/>
+      <c r="I37" t="inlineStr"/>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>113.0</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
         <is>
           <t>الفَلَق</t>
         </is>
       </c>
-      <c r="J37" t="n">
-        <v>5</v>
-      </c>
-      <c r="K37" t="inlineStr">
-        <is>
-          <t>حاسد</t>
-        </is>
-      </c>
-      <c r="L37" t="n">
-        <v>0</v>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>شَرِّ</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>شر</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
-        <v>216.5371900826446</v>
+        <v>245.1157024793388</v>
       </c>
       <c r="B38" t="n">
         <v>428.6776859504132</v>
       </c>
       <c r="C38" t="n">
-        <v>245.1157024793388</v>
+        <v>308.8677685950413</v>
       </c>
       <c r="D38" t="n">
         <v>478.1404958677685</v>
@@ -2081,42 +2409,51 @@
         <v>0</v>
       </c>
       <c r="F38" t="n">
-        <v>44</v>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>إِذَا</t>
-        </is>
-      </c>
-      <c r="H38" t="n">
-        <v>113</v>
-      </c>
-      <c r="I38" t="inlineStr">
+        <v>36</v>
+      </c>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>113.0</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
         <is>
           <t>الفَلَق</t>
         </is>
       </c>
-      <c r="J38" t="n">
-        <v>5</v>
-      </c>
-      <c r="K38" t="inlineStr">
-        <is>
-          <t>إذا</t>
-        </is>
-      </c>
-      <c r="L38" t="n">
-        <v>0</v>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>حَاسِدٍ</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>حاسد</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
-        <v>151.6859504132231</v>
+        <v>216.5371900826446</v>
       </c>
       <c r="B39" t="n">
         <v>428.6776859504132</v>
       </c>
       <c r="C39" t="n">
-        <v>216.5371900826446</v>
+        <v>245.1157024793388</v>
       </c>
       <c r="D39" t="n">
         <v>478.1404958677685</v>
@@ -2125,86 +2462,104 @@
         <v>0</v>
       </c>
       <c r="F39" t="n">
-        <v>45</v>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>حَسَدَ</t>
-        </is>
-      </c>
-      <c r="H39" t="n">
-        <v>113</v>
-      </c>
-      <c r="I39" t="inlineStr">
+        <v>37</v>
+      </c>
+      <c r="G39" t="inlineStr"/>
+      <c r="H39" t="inlineStr"/>
+      <c r="I39" t="inlineStr"/>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>113.0</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
         <is>
           <t>الفَلَق</t>
         </is>
       </c>
-      <c r="J39" t="n">
-        <v>5</v>
-      </c>
-      <c r="K39" t="inlineStr">
-        <is>
-          <t>حسد</t>
-        </is>
-      </c>
-      <c r="L39" t="n">
-        <v>0</v>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>إِذَا</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>إذا</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
-        <v>466.0495867768595</v>
+        <v>151.6859504132231</v>
       </c>
       <c r="B40" t="n">
-        <v>586.9586776859503</v>
+        <v>428.6776859504132</v>
       </c>
       <c r="C40" t="n">
-        <v>497.9256198347107</v>
+        <v>216.5371900826446</v>
       </c>
       <c r="D40" t="n">
-        <v>637.5206611570247</v>
+        <v>478.1404958677685</v>
       </c>
       <c r="E40" t="b">
         <v>0</v>
       </c>
       <c r="F40" t="n">
-        <v>46</v>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>قُلۡ</t>
-        </is>
-      </c>
-      <c r="H40" t="n">
-        <v>114</v>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>النَّاس</t>
-        </is>
-      </c>
-      <c r="J40" t="n">
-        <v>1</v>
+        <v>38</v>
+      </c>
+      <c r="G40" t="inlineStr"/>
+      <c r="H40" t="inlineStr"/>
+      <c r="I40" t="inlineStr"/>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>113.0</t>
+        </is>
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>قل</t>
-        </is>
-      </c>
-      <c r="L40" t="n">
-        <v>0</v>
+          <t>الفَلَق</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>حَسَدَ</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>حسد</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
-        <v>413.2892561983471</v>
+        <v>466.0495867768595</v>
       </c>
       <c r="B41" t="n">
         <v>586.9586776859503</v>
       </c>
       <c r="C41" t="n">
-        <v>466.0495867768595</v>
+        <v>497.9256198347107</v>
       </c>
       <c r="D41" t="n">
         <v>637.5206611570247</v>
@@ -2213,42 +2568,51 @@
         <v>0</v>
       </c>
       <c r="F41" t="n">
-        <v>47</v>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>أَعُوذُ</t>
-        </is>
-      </c>
-      <c r="H41" t="n">
-        <v>114</v>
-      </c>
-      <c r="I41" t="inlineStr">
+        <v>39</v>
+      </c>
+      <c r="G41" t="inlineStr"/>
+      <c r="H41" t="inlineStr"/>
+      <c r="I41" t="inlineStr"/>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>114.0</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
         <is>
           <t>النَّاس</t>
         </is>
       </c>
-      <c r="J41" t="n">
-        <v>1</v>
-      </c>
-      <c r="K41" t="inlineStr">
-        <is>
-          <t>أعوذ</t>
-        </is>
-      </c>
-      <c r="L41" t="n">
-        <v>0</v>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>قُلۡ</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>قل</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
-        <v>356.1322314049586</v>
+        <v>413.2892561983471</v>
       </c>
       <c r="B42" t="n">
         <v>586.9586776859503</v>
       </c>
       <c r="C42" t="n">
-        <v>413.2892561983471</v>
+        <v>466.0495867768595</v>
       </c>
       <c r="D42" t="n">
         <v>637.5206611570247</v>
@@ -2257,42 +2621,51 @@
         <v>0</v>
       </c>
       <c r="F42" t="n">
-        <v>48</v>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>بِرَبِّ</t>
-        </is>
-      </c>
-      <c r="H42" t="n">
-        <v>114</v>
-      </c>
-      <c r="I42" t="inlineStr">
+        <v>40</v>
+      </c>
+      <c r="G42" t="inlineStr"/>
+      <c r="H42" t="inlineStr"/>
+      <c r="I42" t="inlineStr"/>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>114.0</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
         <is>
           <t>النَّاس</t>
         </is>
       </c>
-      <c r="J42" t="n">
-        <v>1</v>
-      </c>
-      <c r="K42" t="inlineStr">
-        <is>
-          <t>برب</t>
-        </is>
-      </c>
-      <c r="L42" t="n">
-        <v>0</v>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>أَعُوذُ</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>أعوذ</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
-        <v>283.5867768595041</v>
+        <v>356.1322314049586</v>
       </c>
       <c r="B43" t="n">
         <v>586.9586776859503</v>
       </c>
       <c r="C43" t="n">
-        <v>356.1322314049586</v>
+        <v>413.2892561983471</v>
       </c>
       <c r="D43" t="n">
         <v>637.5206611570247</v>
@@ -2301,42 +2674,51 @@
         <v>0</v>
       </c>
       <c r="F43" t="n">
-        <v>49</v>
-      </c>
-      <c r="G43" t="inlineStr">
-        <is>
-          <t>ٱلنَّاسِ</t>
-        </is>
-      </c>
-      <c r="H43" t="n">
-        <v>114</v>
-      </c>
-      <c r="I43" t="inlineStr">
+        <v>41</v>
+      </c>
+      <c r="G43" t="inlineStr"/>
+      <c r="H43" t="inlineStr"/>
+      <c r="I43" t="inlineStr"/>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>114.0</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
         <is>
           <t>النَّاس</t>
         </is>
       </c>
-      <c r="J43" t="n">
-        <v>1</v>
-      </c>
-      <c r="K43" t="inlineStr">
-        <is>
-          <t>الناس</t>
-        </is>
-      </c>
-      <c r="L43" t="n">
-        <v>0</v>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>بِرَبِّ</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>برب</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>184.6611570247934</v>
+        <v>283.5867768595041</v>
       </c>
       <c r="B44" t="n">
         <v>586.9586776859503</v>
       </c>
       <c r="C44" t="n">
-        <v>246.2148760330578</v>
+        <v>356.1322314049586</v>
       </c>
       <c r="D44" t="n">
         <v>637.5206611570247</v>
@@ -2345,42 +2727,51 @@
         <v>0</v>
       </c>
       <c r="F44" t="n">
-        <v>51</v>
-      </c>
-      <c r="G44" t="inlineStr">
-        <is>
-          <t>مَلِكِ</t>
-        </is>
-      </c>
-      <c r="H44" t="n">
-        <v>114</v>
-      </c>
-      <c r="I44" t="inlineStr">
+        <v>42</v>
+      </c>
+      <c r="G44" t="inlineStr"/>
+      <c r="H44" t="inlineStr"/>
+      <c r="I44" t="inlineStr"/>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>114.0</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
         <is>
           <t>النَّاس</t>
         </is>
       </c>
-      <c r="J44" t="n">
-        <v>2</v>
-      </c>
-      <c r="K44" t="inlineStr">
-        <is>
-          <t>ملك</t>
-        </is>
-      </c>
-      <c r="L44" t="n">
-        <v>0</v>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>1.0</t>
+        </is>
+      </c>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>ٱلنَّاسِ</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>الناس</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>111.0165289256198</v>
+        <v>184.6611570247934</v>
       </c>
       <c r="B45" t="n">
         <v>586.9586776859503</v>
       </c>
       <c r="C45" t="n">
-        <v>184.6611570247934</v>
+        <v>246.2148760330578</v>
       </c>
       <c r="D45" t="n">
         <v>637.5206611570247</v>
@@ -2389,42 +2780,51 @@
         <v>0</v>
       </c>
       <c r="F45" t="n">
-        <v>52</v>
-      </c>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>ٱلنَّاسِ</t>
-        </is>
-      </c>
-      <c r="H45" t="n">
-        <v>114</v>
-      </c>
-      <c r="I45" t="inlineStr">
+        <v>43</v>
+      </c>
+      <c r="G45" t="inlineStr"/>
+      <c r="H45" t="inlineStr"/>
+      <c r="I45" t="inlineStr"/>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>114.0</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
         <is>
           <t>النَّاس</t>
         </is>
       </c>
-      <c r="J45" t="n">
-        <v>2</v>
-      </c>
-      <c r="K45" t="inlineStr">
-        <is>
-          <t>الناس</t>
-        </is>
-      </c>
-      <c r="L45" t="n">
-        <v>0</v>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>مَلِكِ</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>ملك</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>19.78512396694215</v>
+        <v>111.0165289256198</v>
       </c>
       <c r="B46" t="n">
         <v>586.9586776859503</v>
       </c>
       <c r="C46" t="n">
-        <v>73.64462809917354</v>
+        <v>184.6611570247934</v>
       </c>
       <c r="D46" t="n">
         <v>637.5206611570247</v>
@@ -2433,86 +2833,104 @@
         <v>0</v>
       </c>
       <c r="F46" t="n">
-        <v>54</v>
-      </c>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>إِلَٰهِ</t>
-        </is>
-      </c>
-      <c r="H46" t="n">
-        <v>114</v>
-      </c>
-      <c r="I46" t="inlineStr">
+        <v>44</v>
+      </c>
+      <c r="G46" t="inlineStr"/>
+      <c r="H46" t="inlineStr"/>
+      <c r="I46" t="inlineStr"/>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>114.0</t>
+        </is>
+      </c>
+      <c r="K46" t="inlineStr">
         <is>
           <t>النَّاس</t>
         </is>
       </c>
-      <c r="J46" t="n">
-        <v>3</v>
-      </c>
-      <c r="K46" t="inlineStr">
-        <is>
-          <t>إله</t>
-        </is>
-      </c>
-      <c r="L46" t="n">
-        <v>0</v>
+      <c r="L46" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
+      </c>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>ٱلنَّاسِ</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>الناس</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="n">
-        <v>422.0826446280992</v>
+        <v>19.78512396694215</v>
       </c>
       <c r="B47" t="n">
+        <v>586.9586776859503</v>
+      </c>
+      <c r="C47" t="n">
+        <v>73.64462809917354</v>
+      </c>
+      <c r="D47" t="n">
         <v>637.5206611570247</v>
       </c>
-      <c r="C47" t="n">
-        <v>497.9256198347107</v>
-      </c>
-      <c r="D47" t="n">
-        <v>691.3801652892562</v>
-      </c>
       <c r="E47" t="b">
         <v>0</v>
       </c>
       <c r="F47" t="n">
-        <v>55</v>
-      </c>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>ٱلنَّاسِ</t>
-        </is>
-      </c>
-      <c r="H47" t="n">
-        <v>114</v>
-      </c>
-      <c r="I47" t="inlineStr">
+        <v>45</v>
+      </c>
+      <c r="G47" t="inlineStr"/>
+      <c r="H47" t="inlineStr"/>
+      <c r="I47" t="inlineStr"/>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>114.0</t>
+        </is>
+      </c>
+      <c r="K47" t="inlineStr">
         <is>
           <t>النَّاس</t>
         </is>
       </c>
-      <c r="J47" t="n">
-        <v>3</v>
-      </c>
-      <c r="K47" t="inlineStr">
-        <is>
-          <t>الناس</t>
-        </is>
-      </c>
-      <c r="L47" t="n">
-        <v>0</v>
+      <c r="L47" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>إِلَٰهِ</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>إله</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="n">
-        <v>338.5454545454545</v>
+        <v>422.0826446280992</v>
       </c>
       <c r="B48" t="n">
         <v>637.5206611570247</v>
       </c>
       <c r="C48" t="n">
-        <v>385.8099173553719</v>
+        <v>497.9256198347107</v>
       </c>
       <c r="D48" t="n">
         <v>691.3801652892562</v>
@@ -2521,42 +2939,51 @@
         <v>0</v>
       </c>
       <c r="F48" t="n">
-        <v>57</v>
-      </c>
-      <c r="G48" t="inlineStr">
-        <is>
-          <t>مِن</t>
-        </is>
-      </c>
-      <c r="H48" t="n">
-        <v>114</v>
-      </c>
-      <c r="I48" t="inlineStr">
+        <v>46</v>
+      </c>
+      <c r="G48" t="inlineStr"/>
+      <c r="H48" t="inlineStr"/>
+      <c r="I48" t="inlineStr"/>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>114.0</t>
+        </is>
+      </c>
+      <c r="K48" t="inlineStr">
         <is>
           <t>النَّاس</t>
         </is>
       </c>
-      <c r="J48" t="n">
-        <v>4</v>
-      </c>
-      <c r="K48" t="inlineStr">
-        <is>
-          <t>من</t>
-        </is>
-      </c>
-      <c r="L48" t="n">
-        <v>0</v>
+      <c r="L48" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
+      </c>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>ٱلنَّاسِ</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>الناس</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="n">
-        <v>296.7768595041322</v>
+        <v>338.5454545454545</v>
       </c>
       <c r="B49" t="n">
         <v>637.5206611570247</v>
       </c>
       <c r="C49" t="n">
-        <v>338.5454545454545</v>
+        <v>385.8099173553719</v>
       </c>
       <c r="D49" t="n">
         <v>691.3801652892562</v>
@@ -2565,42 +2992,51 @@
         <v>0</v>
       </c>
       <c r="F49" t="n">
-        <v>58</v>
-      </c>
-      <c r="G49" t="inlineStr">
-        <is>
-          <t>شَرِّ</t>
-        </is>
-      </c>
-      <c r="H49" t="n">
-        <v>114</v>
-      </c>
-      <c r="I49" t="inlineStr">
+        <v>47</v>
+      </c>
+      <c r="G49" t="inlineStr"/>
+      <c r="H49" t="inlineStr"/>
+      <c r="I49" t="inlineStr"/>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>114.0</t>
+        </is>
+      </c>
+      <c r="K49" t="inlineStr">
         <is>
           <t>النَّاس</t>
         </is>
       </c>
-      <c r="J49" t="n">
-        <v>4</v>
-      </c>
-      <c r="K49" t="inlineStr">
-        <is>
-          <t>شر</t>
-        </is>
-      </c>
-      <c r="L49" t="n">
-        <v>0</v>
+      <c r="L49" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>مِن</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>من</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="n">
-        <v>200.0495867768595</v>
+        <v>296.7768595041322</v>
       </c>
       <c r="B50" t="n">
         <v>637.5206611570247</v>
       </c>
       <c r="C50" t="n">
-        <v>296.7768595041322</v>
+        <v>338.5454545454545</v>
       </c>
       <c r="D50" t="n">
         <v>691.3801652892562</v>
@@ -2609,42 +3045,51 @@
         <v>0</v>
       </c>
       <c r="F50" t="n">
-        <v>59</v>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>ٱلۡوَسۡوَاسِ</t>
-        </is>
-      </c>
-      <c r="H50" t="n">
-        <v>114</v>
-      </c>
-      <c r="I50" t="inlineStr">
+        <v>48</v>
+      </c>
+      <c r="G50" t="inlineStr"/>
+      <c r="H50" t="inlineStr"/>
+      <c r="I50" t="inlineStr"/>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>114.0</t>
+        </is>
+      </c>
+      <c r="K50" t="inlineStr">
         <is>
           <t>النَّاس</t>
         </is>
       </c>
-      <c r="J50" t="n">
-        <v>4</v>
-      </c>
-      <c r="K50" t="inlineStr">
-        <is>
-          <t>الوسواس</t>
-        </is>
-      </c>
-      <c r="L50" t="n">
-        <v>0</v>
+      <c r="L50" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>شَرِّ</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>شر</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="n">
-        <v>119.8099173553719</v>
+        <v>200.0495867768595</v>
       </c>
       <c r="B51" t="n">
         <v>637.5206611570247</v>
       </c>
       <c r="C51" t="n">
-        <v>200.0495867768595</v>
+        <v>296.7768595041322</v>
       </c>
       <c r="D51" t="n">
         <v>691.3801652892562</v>
@@ -2653,42 +3098,51 @@
         <v>0</v>
       </c>
       <c r="F51" t="n">
-        <v>60</v>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>ٱلۡخَنَّاسِ</t>
-        </is>
-      </c>
-      <c r="H51" t="n">
-        <v>114</v>
-      </c>
-      <c r="I51" t="inlineStr">
+        <v>49</v>
+      </c>
+      <c r="G51" t="inlineStr"/>
+      <c r="H51" t="inlineStr"/>
+      <c r="I51" t="inlineStr"/>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>114.0</t>
+        </is>
+      </c>
+      <c r="K51" t="inlineStr">
         <is>
           <t>النَّاس</t>
         </is>
       </c>
-      <c r="J51" t="n">
-        <v>4</v>
-      </c>
-      <c r="K51" t="inlineStr">
-        <is>
-          <t>الخناس</t>
-        </is>
-      </c>
-      <c r="L51" t="n">
-        <v>0</v>
+      <c r="L51" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="M51" t="inlineStr">
+        <is>
+          <t>ٱلۡوَسۡوَاسِ</t>
+        </is>
+      </c>
+      <c r="N51" t="inlineStr">
+        <is>
+          <t>الوسواس</t>
+        </is>
+      </c>
+      <c r="O51" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="n">
-        <v>16.48760330578512</v>
+        <v>119.8099173553719</v>
       </c>
       <c r="B52" t="n">
         <v>637.5206611570247</v>
       </c>
       <c r="C52" t="n">
-        <v>82.43801652892562</v>
+        <v>200.0495867768595</v>
       </c>
       <c r="D52" t="n">
         <v>691.3801652892562</v>
@@ -2697,86 +3151,104 @@
         <v>0</v>
       </c>
       <c r="F52" t="n">
-        <v>62</v>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>ٱلَّذِي</t>
-        </is>
-      </c>
-      <c r="H52" t="n">
-        <v>114</v>
-      </c>
-      <c r="I52" t="inlineStr">
+        <v>50</v>
+      </c>
+      <c r="G52" t="inlineStr"/>
+      <c r="H52" t="inlineStr"/>
+      <c r="I52" t="inlineStr"/>
+      <c r="J52" t="inlineStr">
+        <is>
+          <t>114.0</t>
+        </is>
+      </c>
+      <c r="K52" t="inlineStr">
         <is>
           <t>النَّاس</t>
         </is>
       </c>
-      <c r="J52" t="n">
-        <v>5</v>
-      </c>
-      <c r="K52" t="inlineStr">
-        <is>
-          <t>الذي</t>
-        </is>
-      </c>
-      <c r="L52" t="n">
-        <v>0</v>
+      <c r="L52" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="M52" t="inlineStr">
+        <is>
+          <t>ٱلۡخَنَّاسِ</t>
+        </is>
+      </c>
+      <c r="N52" t="inlineStr">
+        <is>
+          <t>الخناس</t>
+        </is>
+      </c>
+      <c r="O52" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="n">
-        <v>315.4628099173553</v>
+        <v>16.48760330578512</v>
       </c>
       <c r="B53" t="n">
+        <v>637.5206611570247</v>
+      </c>
+      <c r="C53" t="n">
+        <v>82.43801652892562</v>
+      </c>
+      <c r="D53" t="n">
         <v>691.3801652892562</v>
       </c>
-      <c r="C53" t="n">
-        <v>400.099173553719</v>
-      </c>
-      <c r="D53" t="n">
-        <v>743.0413223140495</v>
-      </c>
       <c r="E53" t="b">
         <v>0</v>
       </c>
       <c r="F53" t="n">
-        <v>63</v>
-      </c>
-      <c r="G53" t="inlineStr">
-        <is>
-          <t>يُوَسۡوِسُ</t>
-        </is>
-      </c>
-      <c r="H53" t="n">
-        <v>114</v>
-      </c>
-      <c r="I53" t="inlineStr">
+        <v>51</v>
+      </c>
+      <c r="G53" t="inlineStr"/>
+      <c r="H53" t="inlineStr"/>
+      <c r="I53" t="inlineStr"/>
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>114.0</t>
+        </is>
+      </c>
+      <c r="K53" t="inlineStr">
         <is>
           <t>النَّاس</t>
         </is>
       </c>
-      <c r="J53" t="n">
-        <v>5</v>
-      </c>
-      <c r="K53" t="inlineStr">
-        <is>
-          <t>يوسوس</t>
-        </is>
-      </c>
-      <c r="L53" t="n">
-        <v>0</v>
+      <c r="L53" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="M53" t="inlineStr">
+        <is>
+          <t>ٱلَّذِي</t>
+        </is>
+      </c>
+      <c r="N53" t="inlineStr">
+        <is>
+          <t>الذي</t>
+        </is>
+      </c>
+      <c r="O53" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="n">
-        <v>291.2809917355372</v>
+        <v>315.4628099173553</v>
       </c>
       <c r="B54" t="n">
         <v>691.3801652892562</v>
       </c>
       <c r="C54" t="n">
-        <v>315.4628099173553</v>
+        <v>400.099173553719</v>
       </c>
       <c r="D54" t="n">
         <v>743.0413223140495</v>
@@ -2785,42 +3257,51 @@
         <v>0</v>
       </c>
       <c r="F54" t="n">
-        <v>64</v>
-      </c>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>فِي</t>
-        </is>
-      </c>
-      <c r="H54" t="n">
-        <v>114</v>
-      </c>
-      <c r="I54" t="inlineStr">
+        <v>52</v>
+      </c>
+      <c r="G54" t="inlineStr"/>
+      <c r="H54" t="inlineStr"/>
+      <c r="I54" t="inlineStr"/>
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>114.0</t>
+        </is>
+      </c>
+      <c r="K54" t="inlineStr">
         <is>
           <t>النَّاس</t>
         </is>
       </c>
-      <c r="J54" t="n">
-        <v>5</v>
-      </c>
-      <c r="K54" t="inlineStr">
-        <is>
-          <t>في</t>
-        </is>
-      </c>
-      <c r="L54" t="n">
-        <v>0</v>
+      <c r="L54" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="M54" t="inlineStr">
+        <is>
+          <t>يُوَسۡوِسُ</t>
+        </is>
+      </c>
+      <c r="N54" t="inlineStr">
+        <is>
+          <t>يوسوس</t>
+        </is>
+      </c>
+      <c r="O54" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="n">
-        <v>223.1322314049586</v>
+        <v>291.2809917355372</v>
       </c>
       <c r="B55" t="n">
         <v>691.3801652892562</v>
       </c>
       <c r="C55" t="n">
-        <v>291.2809917355372</v>
+        <v>315.4628099173553</v>
       </c>
       <c r="D55" t="n">
         <v>743.0413223140495</v>
@@ -2829,42 +3310,51 @@
         <v>0</v>
       </c>
       <c r="F55" t="n">
-        <v>65</v>
-      </c>
-      <c r="G55" t="inlineStr">
-        <is>
-          <t>صُدُورِ</t>
-        </is>
-      </c>
-      <c r="H55" t="n">
-        <v>114</v>
-      </c>
-      <c r="I55" t="inlineStr">
+        <v>53</v>
+      </c>
+      <c r="G55" t="inlineStr"/>
+      <c r="H55" t="inlineStr"/>
+      <c r="I55" t="inlineStr"/>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>114.0</t>
+        </is>
+      </c>
+      <c r="K55" t="inlineStr">
         <is>
           <t>النَّاس</t>
         </is>
       </c>
-      <c r="J55" t="n">
-        <v>5</v>
-      </c>
-      <c r="K55" t="inlineStr">
-        <is>
-          <t>صدور</t>
-        </is>
-      </c>
-      <c r="L55" t="n">
-        <v>0</v>
+      <c r="L55" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="M55" t="inlineStr">
+        <is>
+          <t>فِي</t>
+        </is>
+      </c>
+      <c r="N55" t="inlineStr">
+        <is>
+          <t>في</t>
+        </is>
+      </c>
+      <c r="O55" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="n">
-        <v>149.4876033057851</v>
+        <v>223.1322314049586</v>
       </c>
       <c r="B56" t="n">
         <v>691.3801652892562</v>
       </c>
       <c r="C56" t="n">
-        <v>223.1322314049586</v>
+        <v>291.2809917355372</v>
       </c>
       <c r="D56" t="n">
         <v>743.0413223140495</v>
@@ -2873,86 +3363,104 @@
         <v>0</v>
       </c>
       <c r="F56" t="n">
-        <v>66</v>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>ٱلنَّاسِ</t>
-        </is>
-      </c>
-      <c r="H56" t="n">
-        <v>114</v>
-      </c>
-      <c r="I56" t="inlineStr">
+        <v>54</v>
+      </c>
+      <c r="G56" t="inlineStr"/>
+      <c r="H56" t="inlineStr"/>
+      <c r="I56" t="inlineStr"/>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>114.0</t>
+        </is>
+      </c>
+      <c r="K56" t="inlineStr">
         <is>
           <t>النَّاس</t>
         </is>
       </c>
-      <c r="J56" t="n">
-        <v>5</v>
-      </c>
-      <c r="K56" t="inlineStr">
-        <is>
-          <t>الناس</t>
-        </is>
-      </c>
-      <c r="L56" t="n">
-        <v>0</v>
+      <c r="L56" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="M56" t="inlineStr">
+        <is>
+          <t>صُدُورِ</t>
+        </is>
+      </c>
+      <c r="N56" t="inlineStr">
+        <is>
+          <t>صدور</t>
+        </is>
+      </c>
+      <c r="O56" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="n">
-        <v>335.2479338842975</v>
+        <v>149.4876033057851</v>
       </c>
       <c r="B57" t="n">
+        <v>691.3801652892562</v>
+      </c>
+      <c r="C57" t="n">
+        <v>223.1322314049586</v>
+      </c>
+      <c r="D57" t="n">
         <v>743.0413223140495</v>
       </c>
-      <c r="C57" t="n">
-        <v>369.3223140495867</v>
-      </c>
-      <c r="D57" t="n">
-        <v>795.8016528925619</v>
-      </c>
       <c r="E57" t="b">
         <v>0</v>
       </c>
       <c r="F57" t="n">
-        <v>67</v>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>مِنَ</t>
-        </is>
-      </c>
-      <c r="H57" t="n">
-        <v>114</v>
-      </c>
-      <c r="I57" t="inlineStr">
+        <v>55</v>
+      </c>
+      <c r="G57" t="inlineStr"/>
+      <c r="H57" t="inlineStr"/>
+      <c r="I57" t="inlineStr"/>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>114.0</t>
+        </is>
+      </c>
+      <c r="K57" t="inlineStr">
         <is>
           <t>النَّاس</t>
         </is>
       </c>
-      <c r="J57" t="n">
-        <v>6</v>
-      </c>
-      <c r="K57" t="inlineStr">
-        <is>
-          <t>من</t>
-        </is>
-      </c>
-      <c r="L57" t="n">
-        <v>0</v>
+      <c r="L57" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="M57" t="inlineStr">
+        <is>
+          <t>ٱلنَّاسِ</t>
+        </is>
+      </c>
+      <c r="N57" t="inlineStr">
+        <is>
+          <t>الناس</t>
+        </is>
+      </c>
+      <c r="O57" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="n">
-        <v>262.702479338843</v>
+        <v>335.2479338842975</v>
       </c>
       <c r="B58" t="n">
         <v>743.0413223140495</v>
       </c>
       <c r="C58" t="n">
-        <v>335.2479338842975</v>
+        <v>369.3223140495867</v>
       </c>
       <c r="D58" t="n">
         <v>795.8016528925619</v>
@@ -2961,42 +3469,51 @@
         <v>0</v>
       </c>
       <c r="F58" t="n">
-        <v>68</v>
-      </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>ٱلۡجِنَّةِ</t>
-        </is>
-      </c>
-      <c r="H58" t="n">
-        <v>114</v>
-      </c>
-      <c r="I58" t="inlineStr">
+        <v>56</v>
+      </c>
+      <c r="G58" t="inlineStr"/>
+      <c r="H58" t="inlineStr"/>
+      <c r="I58" t="inlineStr"/>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>114.0</t>
+        </is>
+      </c>
+      <c r="K58" t="inlineStr">
         <is>
           <t>النَّاس</t>
         </is>
       </c>
-      <c r="J58" t="n">
-        <v>6</v>
-      </c>
-      <c r="K58" t="inlineStr">
-        <is>
-          <t>الجنة</t>
-        </is>
-      </c>
-      <c r="L58" t="n">
-        <v>0</v>
+      <c r="L58" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="M58" t="inlineStr">
+        <is>
+          <t>مِنَ</t>
+        </is>
+      </c>
+      <c r="N58" t="inlineStr">
+        <is>
+          <t>من</t>
+        </is>
+      </c>
+      <c r="O58" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="n">
-        <v>182.4628099173553</v>
+        <v>262.702479338843</v>
       </c>
       <c r="B59" t="n">
         <v>743.0413223140495</v>
       </c>
       <c r="C59" t="n">
-        <v>262.702479338843</v>
+        <v>335.2479338842975</v>
       </c>
       <c r="D59" t="n">
         <v>795.8016528925619</v>
@@ -3005,23 +3522,93 @@
         <v>0</v>
       </c>
       <c r="F59" t="n">
-        <v>69</v>
-      </c>
-      <c r="G59" t="inlineStr">
-        <is>
-          <t>وَٱلنَّاسِ</t>
-        </is>
-      </c>
+        <v>57</v>
+      </c>
+      <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr"/>
-      <c r="J59" t="inlineStr"/>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>114.0</t>
+        </is>
+      </c>
       <c r="K59" t="inlineStr">
         <is>
+          <t>النَّاس</t>
+        </is>
+      </c>
+      <c r="L59" t="inlineStr">
+        <is>
+          <t>6.0</t>
+        </is>
+      </c>
+      <c r="M59" t="inlineStr">
+        <is>
+          <t>ٱلۡجِنَّةِ</t>
+        </is>
+      </c>
+      <c r="N59" t="inlineStr">
+        <is>
+          <t>الجنة</t>
+        </is>
+      </c>
+      <c r="O59" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>182.4628099173553</v>
+      </c>
+      <c r="B60" t="n">
+        <v>743.0413223140495</v>
+      </c>
+      <c r="C60" t="n">
+        <v>262.702479338843</v>
+      </c>
+      <c r="D60" t="n">
+        <v>795.8016528925619</v>
+      </c>
+      <c r="E60" t="b">
+        <v>0</v>
+      </c>
+      <c r="F60" t="n">
+        <v>58</v>
+      </c>
+      <c r="G60" t="inlineStr"/>
+      <c r="H60" t="inlineStr"/>
+      <c r="I60" t="inlineStr"/>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="K60" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="L60" t="inlineStr">
+        <is>
+          <t>nan</t>
+        </is>
+      </c>
+      <c r="M60" t="inlineStr">
+        <is>
+          <t>وَٱلنَّاسِ</t>
+        </is>
+      </c>
+      <c r="N60" t="inlineStr">
+        <is>
           <t>والناس</t>
         </is>
       </c>
-      <c r="L59" t="n">
-        <v>0</v>
+      <c r="O60" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -3986,4 +4573,110 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>x1</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>y1</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>x2</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>y2</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>363.8185745140389</v>
+      </c>
+      <c r="B2" t="n">
+        <v>113.2148760330578</v>
+      </c>
+      <c r="C2" t="n">
+        <v>403.396694214876</v>
+      </c>
+      <c r="D2" t="n">
+        <v>161.5785123966942</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>349.4427645788337</v>
+      </c>
+      <c r="B3" t="n">
+        <v>113.2148760330578</v>
+      </c>
+      <c r="C3" t="n">
+        <v>363.8185745140389</v>
+      </c>
+      <c r="D3" t="n">
+        <v>161.5785123966942</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>327.5537190082644</v>
+      </c>
+      <c r="B4" t="n">
+        <v>113.2148760330578</v>
+      </c>
+      <c r="C4" t="n">
+        <v>349.4427645788337</v>
+      </c>
+      <c r="D4" t="n">
+        <v>161.5785123966942</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>350.548596112311</v>
+      </c>
+      <c r="B5" t="n">
+        <v>113.2148760330578</v>
+      </c>
+      <c r="C5" t="n">
+        <v>403.396694214876</v>
+      </c>
+      <c r="D5" t="n">
+        <v>161.5785123966942</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>327.5537190082644</v>
+      </c>
+      <c r="B6" t="n">
+        <v>113.2148760330578</v>
+      </c>
+      <c r="C6" t="n">
+        <v>350.548596112311</v>
+      </c>
+      <c r="D6" t="n">
+        <v>161.5785123966942</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>